<commit_message>
SkyG Speed 90B C6B-7: 320 mm tube, four wing screws in steel cup washers, GPS cradle
</commit_message>
<xml_diff>
--- a/c6b/downloads/C6B/SkyG-Speed-90B-C6B-7-BOM.xlsx
+++ b/c6b/downloads/C6B/SkyG-Speed-90B-C6B-7-BOM.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Printed parts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Order list (BOM)'!$A$4:$J$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Order list (BOM)'!$A$4:$J$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Printed parts'!$A$4:$F$32</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1445,7 +1445,7 @@
         <v>4</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
@@ -1459,7 +1459,7 @@
       </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t>Wing mount, front screw (x = wing LE + 16)</t>
+          <t>Wing mount, front screws (x = wing LE + 16), one in each wing half 6.5 mm from the centreline, in steel cup washers</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
@@ -1488,10 +1488,10 @@
         </is>
       </c>
       <c r="D25" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>Saddle nut pockets</t>
+          <t>Wing screw nuts, two in each bonded nut bar</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -2335,7 +2335,7 @@
         <v>4</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
@@ -2349,7 +2349,7 @@
       </c>
       <c r="H44" s="8" t="inlineStr">
         <is>
-          <t>Wing mount, rear screw (x = wing LE + 58, ahead of the aileron horns)</t>
+          <t>Wing mount, rear screws (x = wing LE + 58, ahead of the aileron horns), one in each wing half 6.5 mm from the centreline, in steel cup washers</t>
         </is>
       </c>
       <c r="I44" s="7" t="inlineStr">
@@ -2365,7 +2365,7 @@
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
-        <v>54</v>
+        <v>83</v>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
@@ -2374,28 +2374,28 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>M2 x 6 countersunk screws (motor plate)</t>
+          <t>Steel cup washer M3 (countersunk finishing washer)</t>
         </is>
       </c>
       <c r="D45" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E45" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E45" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>M2 x 6 countersunk (DIN 965), steel</t>
+          <t>Countersunk finishing (cup) washer for M3, about 8 mm OD x 1.8 mm, steel black oxide (or A2 stainless)</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>M2x6 countersunk screws</t>
+          <t>M3 countersunk finishing washer black</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>Motor plate M1: one each side, flush in a printed countersunk washer (CW) in a 5 mm counterbore in the tail module's side, into the plate's lugs (in pockets in the seat ring)</t>
+          <t>Under the four M3 wing screws, flush in the recesses in the wing top</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
@@ -2405,43 +2405,43 @@
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>C6B-6 (owner 2026-10-08): screwed in instead of bonded; the plate comes out for a different motor</t>
+          <t>Owner 2026-10-08: steel cup washers on the wing and hatch screws (removed most often); the recess is 8.3 mm x 1.85 mm: check your washers</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n">
-        <v>55</v>
+        <v>84</v>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Consumables</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Servo strap / zip tie + foam tape</t>
+          <t>Steel cup washer M2 (countersunk finishing washer)</t>
         </is>
       </c>
       <c r="D46" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E46" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E46" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>3 mm zip tie or 6 mm strap; double-sided foam tape</t>
+          <t>Countersunk finishing (cup) washer for M2, about 6 mm OD x 1.4 mm, steel black oxide (or A2 stainless)</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>Small zip ties + servo tape</t>
+          <t>M2 countersunk finishing washer black</t>
         </is>
       </c>
       <c r="H46" s="8" t="inlineStr">
         <is>
-          <t>All three servos: foam tape on the bottom skin through the floor cut-outs, strap over the case</t>
+          <t>Under the two M2 hatch screws, flush in the recesses in the hatch cover</t>
         </is>
       </c>
       <c r="I46" s="7" t="inlineStr">
@@ -2451,43 +2451,43 @@
       </c>
       <c r="J46" s="8" t="inlineStr">
         <is>
-          <t>Removable: the servos come out for motor service</t>
+          <t>Owner 2026-10-08; the recess is 6.3 mm x 1.45 mm: check your washers</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Steel rod 1.5 mm</t>
+          <t>M2 x 6 countersunk screws (motor plate)</t>
         </is>
       </c>
       <c r="D47" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E47" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>1.5 mm music wire or silver steel, &gt;= 270 mm (2 x 132 mm)</t>
+          <t>M2 x 6 countersunk (DIN 965), steel</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>Music wire 1.5 mm</t>
+          <t>M2x6 countersunk screws</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>Aileron hinge pin + spine on the hinge axis (y 82-214)</t>
+          <t>Motor plate M1: one each side, flush in a printed countersunk washer (CW) in a 5 mm counterbore in the tail module's side, into the plate's lugs (in pockets in the seat ring)</t>
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr">
@@ -2497,89 +2497,89 @@
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>Pushed in from the wingtip through the tip bore, the aileron and the two wing knuckles; bonded in the aileron with thin CA through its 3 glue holes, free in the knuckles and the tip. Plug the tip hole</t>
+          <t>C6B-6 (owner 2026-10-08): screwed in instead of bonded; the plate comes out for a different motor</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>Video option (DJI)</t>
+          <t>Consumables</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>DJI O4 Air Unit (Lite)</t>
+          <t>Servo strap / zip tie + foam tape</t>
         </is>
       </c>
       <c r="D48" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E48" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>DJI O4 Air Unit (8.2 g with camera): camera 13.44 x 12.36 x 16.5 mm in a 14 x 20 mm mount, module 30 x 30 x 6 mm (4 x d2.6 on 25.5 mm), 3.7-13.2 V</t>
+          <t>3 mm zip tie or 6 mm strap; double-sided foam tape</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>DJI O4 Air Unit</t>
+          <t>Small zip ties + servo tape</t>
         </is>
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>N0O or N0OD nose (camera + module)</t>
+          <t>All three servos: foam tape on the bottom skin through the floor cut-outs, strap over the case</t>
         </is>
       </c>
       <c r="I48" s="7" t="inlineStr">
         <is>
-          <t>Option</t>
-        </is>
-      </c>
-      <c r="J48" s="9" t="inlineStr">
-        <is>
-          <t>https://www.dji.com/o4-air-unit/specs (dimensions: O4 Air Unit Series User Manual v1.0, sec. 1.2) - replaces the micro camera + VTX; power from the SpeedyBee Vv pad set to the servo BEC (6 V jumper); needs airflow (shuts down after minutes on the bench)</t>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="J48" s="8" t="inlineStr">
+        <is>
+          <t>Removable: the servos come out for motor service</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Video option (DJI)</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>M2 x 5 pan head (O4 camera mount)</t>
+          <t>Steel rod 1.5 mm</t>
         </is>
       </c>
       <c r="D49" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>M2 x 5 pan head (or the screws supplied with the camera)</t>
+          <t>1.5 mm music wire or silver steel, &gt;= 270 mm (2 x 132 mm)</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>M2x5 pan head screws</t>
+          <t>Music wire 1.5 mm</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>N0O / N0OD side bosses into the camera mount</t>
+          <t>Aileron hinge pin + spine on the hinge axis (y 82-214)</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
@@ -2589,13 +2589,13 @@
       </c>
       <c r="J49" s="5" t="inlineStr">
         <is>
-          <t>At most 3.1 mm into the mount's d1.65 holes; fore-aft slots +-1 mm</t>
+          <t>Pushed in from the wingtip through the tip bore, the aileron and the two wing knuckles; bonded in the aileron with thin CA through its 3 glue holes, free in the knuckles and the tip. Plug the tip hole</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
@@ -2604,7 +2604,7 @@
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>Foam strip + tape (O4 module)</t>
+          <t>DJI O4 Air Unit (Lite)</t>
         </is>
       </c>
       <c r="D50" s="7" t="n">
@@ -2615,33 +2615,33 @@
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>2 x 1 mm foam strip, 25 mm; Kapton or aluminium tape</t>
+          <t>DJI O4 Air Unit (8.2 g with camera): camera 13.44 x 12.36 x 16.5 mm in a 14 x 20 mm mount, module 30 x 30 x 6 mm (4 x d2.6 on 25.5 mm), 3.7-13.2 V</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>Double-sided foam tape, Kapton tape</t>
+          <t>DJI O4 Air Unit</t>
         </is>
       </c>
       <c r="H50" s="8" t="inlineStr">
         <is>
-          <t>Module retention in the nose duct</t>
+          <t>N0O or N0OD nose (camera + module)</t>
         </is>
       </c>
       <c r="I50" s="7" t="inlineStr">
         <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="J50" s="8" t="inlineStr">
-        <is>
-          <t>Foam strip in the top groove, tape over the rear edge; nothing may cover the module's faces (they are the cooling surfaces)</t>
+          <t>Option</t>
+        </is>
+      </c>
+      <c r="J50" s="9" t="inlineStr">
+        <is>
+          <t>https://www.dji.com/o4-air-unit/specs (dimensions: O4 Air Unit Series User Manual v1.0, sec. 1.2) - replaces the micro camera + VTX; power from the SpeedyBee Vv pad set to the servo BEC (6 V jumper); needs airflow (shuts down after minutes on the bench)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
@@ -2650,28 +2650,28 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>O4 3-in-1 lead extension</t>
+          <t>M2 x 5 pan head (O4 camera mount)</t>
         </is>
       </c>
       <c r="D51" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>~200 mm, power + UART, plug at the nose joint</t>
+          <t>M2 x 5 pan head (or the screws supplied with the camera)</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>Silicone wire + JST-SH / matching plug</t>
+          <t>M2x5 pan head screws</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>Nose to the flight controller in the wing bay</t>
+          <t>N0O / N0OD side bosses into the camera mount</t>
         </is>
       </c>
       <c r="I51" s="4" t="inlineStr">
@@ -2681,22 +2681,22 @@
       </c>
       <c r="J51" s="5" t="inlineStr">
         <is>
-          <t>MSP DisplayPort OSD on a spare SpeedyBee UART</t>
+          <t>At most 3.1 mm into the mount's d1.65 holes; fore-aft slots +-1 mm</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Consumables</t>
+          <t>Video option (DJI)</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>Vent tape</t>
+          <t>Foam strip + tape (O4 module)</t>
         </is>
       </c>
       <c r="D52" s="7" t="n">
@@ -2707,17 +2707,17 @@
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>Thin smooth tape (e.g. 3M 471 or Kapton), 15 mm</t>
+          <t>2 x 1 mm foam strip, 25 mm; Kapton or aluminium tape</t>
         </is>
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>Vinyl or Kapton tape</t>
+          <t>Double-sided foam tape, Kapton tape</t>
         </is>
       </c>
       <c r="H52" s="8" t="inlineStr">
         <is>
-          <t>Over the nose belly inlet, for record passes only (no openings in the tube or the hatch cover on C6B)</t>
+          <t>Module retention in the nose duct</t>
         </is>
       </c>
       <c r="I52" s="7" t="inlineStr">
@@ -2727,22 +2727,22 @@
       </c>
       <c r="J52" s="8" t="inlineStr">
         <is>
-          <t>Never over the DJI nose's duct openings (the module overheats in about a minute without them)</t>
+          <t>Foam strip in the top groove, tape over the rear edge; nothing may cover the module's faces (they are the cooling surfaces)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Controls</t>
+          <t>Video option (DJI)</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>15T servo arms</t>
+          <t>O4 3-in-1 lead extension</t>
         </is>
       </c>
       <c r="D53" s="4" t="n">
@@ -2753,17 +2753,17 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>15T 3.9-4 mm spline arms: two-sided (aileron) with holes at 4.3 mm, one-sided (tail) with a hole at 6.7 mm; C6: holes drilled 1.1 mm and reamed to 1.2 mm for the 1.2 mm Z-bends (no play)</t>
+          <t>~200 mm, power + UART, plug at the nose joint</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>Arms supplied with the ES9052MD (drill a 0.85 mm hole at the radius if missing) or a KST X06 arm set</t>
+          <t>Silicone wire + JST-SH / matching plug</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
         <is>
-          <t>Aileron servo: two-sided arm; tail servos: one-sided arms</t>
+          <t>Nose to the flight controller in the wing bay</t>
         </is>
       </c>
       <c r="I53" s="4" t="inlineStr">
@@ -2773,22 +2773,22 @@
       </c>
       <c r="J53" s="5" t="inlineStr">
         <is>
-          <t>Usually supplied with the servos</t>
+          <t>MSP DisplayPort OSD on a spare SpeedyBee UART</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Consumables</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>u.FL extension 1.13 mm, about 250 mm</t>
+          <t>Vent tape</t>
         </is>
       </c>
       <c r="D54" s="7" t="n">
@@ -2799,17 +2799,17 @@
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
-          <t>IPEX / u.FL male to u.FL female 1.13 mm coax, 200-300 mm</t>
+          <t>Thin smooth tape (e.g. 3M 471 or Kapton), 15 mm</t>
         </is>
       </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>u.FL IPEX extension cable 1.13 mm</t>
+          <t>Vinyl or Kapton tape</t>
         </is>
       </c>
       <c r="H54" s="8" t="inlineStr">
         <is>
-          <t>RP1 V2 receiver to the dipole in the fin (W07), u.FL joint at the tail joint</t>
+          <t>Over the nose belly inlet, for record passes only (no openings in the tube or the hatch cover on C6B)</t>
         </is>
       </c>
       <c r="I54" s="7" t="inlineStr">
@@ -2819,43 +2819,43 @@
       </c>
       <c r="J54" s="8" t="inlineStr">
         <is>
-          <t>C6: ELRS dipole in the fin (2026-10-06)</t>
+          <t>Never over the DJI nose's duct openings (the module overheats in about a minute without them)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Controls</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Dupont housings + crimps (1-pin, 4-pin)</t>
+          <t>15T servo arms</t>
         </is>
       </c>
       <c r="D55" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E55" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>2.54 mm Dupont female housings with crimp terminals</t>
+          <t>15T 3.9-4 mm spline arms: two-sided (aileron) with holes at 4.3 mm, one-sided (tail) with a hole at 6.7 mm; C6: holes drilled 1.1 mm and reamed to 1.2 mm for the 1.2 mm Z-bends (no play)</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>Dupont connector kit 2.54 mm</t>
+          <t>Arms supplied with the ES9052MD (drill a 0.85 mm hole at the radius if missing) or a KST X06 arm set</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr">
         <is>
-          <t>ESC signal and GND on S1 (2 x 1-pin), receiver lead on the FC receiver header (4-pin)</t>
+          <t>Aileron servo: two-sided arm; tail servos: one-sided arms</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
@@ -2863,91 +2863,91 @@
           <t>Class</t>
         </is>
       </c>
-      <c r="J55" s="5" t="inlineStr"/>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>Usually supplied with the servos</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t>Carbon-fibre tube 40 x 38 mm</t>
-        </is>
-      </c>
-      <c r="D56" s="7" t="inlineStr">
-        <is>
-          <t>1 (2 m makes 6)</t>
-        </is>
-      </c>
-      <c r="E56" s="7" t="inlineStr">
-        <is>
-          <t>307 mm</t>
-        </is>
+          <t>u.FL extension 1.13 mm, about 250 mm</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t>Roll-wrapped 3K carbon/epoxy, 40.0 mm OD x 38.0 mm ID (1 mm wall), about 178 g/m; straight, round within 0.1 mm</t>
+          <t>IPEX / u.FL male to u.FL female 1.13 mm coax, 200-300 mm</t>
         </is>
       </c>
       <c r="G56" s="8" t="inlineStr">
         <is>
-          <t>Karbon boru 40/38 mm 3K (Kompozit Pazari RFG 2 m; Karbonfiber Boru; PilotTR)</t>
+          <t>u.FL IPEX extension cable 1.13 mm</t>
         </is>
       </c>
       <c r="H56" s="8" t="inlineStr">
         <is>
-          <t>Fuselage x 50-350: camera nose plugs in the front, tail module onto the coupler at the back</t>
+          <t>RP1 V2 receiver to the dipole in the fin (W07), u.FL joint at the tail joint</t>
         </is>
       </c>
       <c r="I56" s="7" t="inlineStr">
         <is>
-          <t>Ordered (owner, 2026-10-07)</t>
+          <t>Class</t>
         </is>
       </c>
       <c r="J56" s="8" t="inlineStr">
         <is>
-          <t>Measure the bore before printing (parameters: fuselage.tube.id); cut length 300 mm, windows and holes from the paper template; 42.8 g as cut</t>
+          <t>C6: ELRS dipole in the fin (2026-10-06)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>M2 x 6 countersunk screws (tube)</t>
+          <t>Dupont housings + crimps (1-pin, 4-pin)</t>
         </is>
       </c>
       <c r="D57" s="4" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E57" s="4" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>M2 x 6 countersunk (DIN 965 / ISO 7046), steel</t>
+          <t>2.54 mm Dupont female housings with crimp terminals</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>M2x6 countersunk screws</t>
+          <t>Dupont connector kit 2.54 mm</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr">
         <is>
-          <t>Flush in a printed countersunk washer (CW; print 14: 8 in the tube, 4 at the tail joint, 2 at the motor plate) in each 5 mm hole in the tube: camera-nose joint (2, 10 mm from the tube's end), equipment tray (4), tail coupler (2, 14 mm from the tube's end; backup to the bond)</t>
+          <t>ESC signal and GND on S1 (2 x 1-pin), receiver lead on the FC receiver header (4-pin)</t>
         </is>
       </c>
       <c r="I57" s="4" t="inlineStr">
@@ -2955,91 +2955,91 @@
           <t>Class</t>
         </is>
       </c>
-      <c r="J57" s="5" t="inlineStr">
-        <is>
-          <t>Owner 2026-10-08: no screw heads standing out; the washer carries the head (no countersink in the 1 mm carbon)</t>
-        </is>
-      </c>
+      <c r="J57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Consumables</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>Structural epoxy</t>
-        </is>
-      </c>
-      <c r="D58" s="7" t="n">
-        <v>1</v>
+          <t>Carbon-fibre tube 40 x 38 mm</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>1 (2 m makes 6)</t>
+        </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>~3 g</t>
+          <t>320 mm</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t>2-part structural epoxy (30-min working time or longer), bonds carbon and PLA; scuff the carbon with 120-grit and clean with alcohol first</t>
+          <t>Roll-wrapped 3K carbon/epoxy, 40.0 mm OD x 38.0 mm ID (1 mm wall), about 178 g/m; straight, round within 0.1 mm</t>
         </is>
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>e.g. UHU Plus Endfest 300, Loctite EA 3430 or laminating epoxy thickened with cotton flock</t>
+          <t>Karbon boru 40/38 mm 3K (Kompozit Pazari RFG 2 m; Karbonfiber Boru; PilotTR)</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>Nut bars, hatch lips, duct inserts, tail coupler and the wing saddle into / onto the tube</t>
+          <t>Fuselage x 50-350: camera nose plugs in the front, tail module onto the coupler at the back</t>
         </is>
       </c>
       <c r="I58" s="7" t="inlineStr">
         <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="J58" s="8" t="inlineStr"/>
+          <t>Ordered (owner, 2026-10-07)</t>
+        </is>
+      </c>
+      <c r="J58" s="8" t="inlineStr">
+        <is>
+          <t>Measure the bore before printing (parameters: fuselage.tube.id); cut length 300 mm, windows and holes from the paper template; 42.8 g as cut</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Consumables</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Thin CA</t>
+          <t>M2 x 6 countersunk screws (tube)</t>
         </is>
       </c>
       <c r="D59" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t>~1 g</t>
-        </is>
+        <v>12</v>
+      </c>
+      <c r="E59" s="4" t="n">
+        <v>8</v>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Thin cyanoacrylate</t>
+          <t>M2 x 6 countersunk (DIN 965 / ISO 7046), steel</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>Thin CA glue</t>
+          <t>M2x6 countersunk screws</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr">
         <is>
-          <t>Seal every cut edge and hole in the carbon tube</t>
+          <t>Flush in a printed countersunk washer (CW; print 14: 8 in the tube, 4 at the tail joint, 2 at the motor plate) in each 5 mm hole in the tube: camera-nose joint (2, 10 mm from the tube's end), equipment tray (4), tail coupler (2, 40 deg above the side line, 12 mm from the tube's end; backup to the bond)</t>
         </is>
       </c>
       <c r="I59" s="4" t="inlineStr">
@@ -3049,22 +3049,22 @@
       </c>
       <c r="J59" s="5" t="inlineStr">
         <is>
-          <t>Carbon conducts: a frayed edge can cut through a wire's insulation and short it</t>
+          <t>Owner 2026-10-08: no screw heads standing out; the washer carries the head (no countersink in the 1 mm carbon)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Tools</t>
+          <t>Consumables</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>Diamond cut-off discs + dust protection</t>
+          <t>Structural epoxy</t>
         </is>
       </c>
       <c r="D60" s="7" t="n">
@@ -3072,68 +3072,66 @@
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>~3 g</t>
         </is>
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>Rotary-tool diamond cut-off discs (or reinforced abrasive), fine file, FFP3 mask, eye protection, vacuum at the disc or cut wet</t>
+          <t>2-part structural epoxy (30-min working time or longer), bonds carbon and PLA; scuff the carbon with 120-grit and clean with alcohol first</t>
         </is>
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>Dremel 545 diamond disc or equivalent</t>
+          <t>e.g. UHU Plus Endfest 300, Loctite EA 3430 or laminating epoxy thickened with cotton flock</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr">
         <is>
-          <t>Cutting the tube to length and its windows</t>
+          <t>Nut bars, hatch lips, duct inserts, tail coupler and the wing saddle into / onto the tube</t>
         </is>
       </c>
       <c r="I60" s="7" t="inlineStr">
         <is>
-          <t>Owner has a Dremel</t>
-        </is>
-      </c>
-      <c r="J60" s="8" t="inlineStr">
-        <is>
-          <t>Carbon dust is a lung irritant and conductive (keep it off electronics)</t>
-        </is>
-      </c>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="J60" s="8" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Consumables</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>M2 x 6 countersunk screws (hatch)</t>
+          <t>Thin CA</t>
         </is>
       </c>
       <c r="D61" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="E61" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>~1 g</t>
+        </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>M2 x 6 countersunk (DIN 965), steel</t>
+          <t>Thin cyanoacrylate</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>M2x6 countersunk screws</t>
+          <t>Thin CA glue</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr">
         <is>
-          <t>Front hatch cover, one at each end, into the bosses under the bonded lips</t>
+          <t>Seal every cut edge and hole in the carbon tube</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
@@ -3143,155 +3141,153 @@
       </c>
       <c r="J61" s="5" t="inlineStr">
         <is>
-          <t>C6B-4 (owner): no magnets</t>
+          <t>Carbon conducts: a frayed edge can cut through a wire's insulation and short it</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Avionics</t>
+          <t>Tools</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t>USB-C extension with socket</t>
+          <t>Diamond cut-off discs + dust protection</t>
         </is>
       </c>
       <c r="D62" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E62" s="7" t="n">
-        <v>1</v>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>USB-C female socket board or panel-mount socket (about 10 x 8 mm) on a 150 mm USB-C extension, thin cable</t>
+          <t>Rotary-tool diamond cut-off discs (or reinforced abrasive), fine file, FFP3 mask, eye protection, vacuum at the disc or cut wet</t>
         </is>
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>USB-C female panel mount extension 15 cm</t>
+          <t>Dremel 545 diamond disc or equivalent</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr">
         <is>
-          <t>FC USB-C to the socket holder on the tray under the hatch cover (left of the GPS lead)</t>
+          <t>Cutting the tube to length and its windows</t>
         </is>
       </c>
       <c r="I62" s="7" t="inlineStr">
         <is>
-          <t>Class</t>
+          <t>Owner has a Dremel</t>
         </is>
       </c>
       <c r="J62" s="8" t="inlineStr">
         <is>
-          <t>C6B-4: FC access for setup, parameters and logs with the hatch cover off</t>
+          <t>Carbon dust is a lung irritant and conductive (keep it off electronics)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Consumables</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Filament PLA-CF</t>
+          <t>M2 x 6 countersunk screws (hatch)</t>
         </is>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E63" s="4" t="inlineStr">
-        <is>
-          <t>94 g</t>
-        </is>
+        <v>4</v>
+      </c>
+      <c r="E63" s="4" t="n">
+        <v>2</v>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Bambu PLA-CF 1 kg (hardened-steel nozzle)</t>
+          <t>M2 x 6 countersunk (DIN 965), steel</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>Bambu PLA-CF 1 kg (hardened-steel nozzle)</t>
+          <t>M2x6 countersunk screws</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr">
         <is>
-          <t>Wing halves WR/WL (2 walls, 8 % gyroid)</t>
+          <t>Front hatch cover, one at each end, into the bosses under the bonded lips</t>
         </is>
       </c>
       <c r="I63" s="4" t="inlineStr">
         <is>
-          <t>Bambu profile</t>
+          <t>Class</t>
         </is>
       </c>
       <c r="J63" s="5" t="inlineStr">
         <is>
-          <t>C6B per-part filaments (design/MATERIALS-NOTES.md); one aircraft with the N0M nose</t>
+          <t>C6B-4 (owner): no magnets</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>Consumables</t>
+          <t>Avionics</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t>Filament PETG-CF</t>
+          <t>USB-C extension with socket</t>
         </is>
       </c>
       <c r="D64" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E64" s="7" t="inlineStr">
-        <is>
-          <t>53 g</t>
-        </is>
+      <c r="E64" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t>Bambu PETG-CF 1 kg (hardened-steel nozzle)</t>
+          <t>USB-C female socket board or panel-mount socket (about 10 x 8 mm) on a 150 mm USB-C extension, thin cable</t>
         </is>
       </c>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t>Bambu PETG-CF 1 kg (hardened-steel nozzle)</t>
+          <t>USB-C female panel mount extension 15 cm</t>
         </is>
       </c>
       <c r="H64" s="8" t="inlineStr">
         <is>
-          <t>Ailerons, equipment tray, tail coupler, nut bars, hatch lips, duct inserts, motor plate, spinner</t>
+          <t>FC USB-C to the socket holder on the tray under the hatch cover (left of the GPS lead)</t>
         </is>
       </c>
       <c r="I64" s="7" t="inlineStr">
         <is>
-          <t>Bambu profile</t>
+          <t>Class</t>
         </is>
       </c>
       <c r="J64" s="8" t="inlineStr">
         <is>
-          <t>C6B per-part filaments (design/MATERIALS-NOTES.md); one aircraft with the N0M nose</t>
+          <t>C6B-4: FC access for setup, parameters and logs with the hatch cover off</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
@@ -3300,7 +3296,7 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Filament ASA</t>
+          <t>Filament PLA-CF</t>
         </is>
       </c>
       <c r="D65" s="4" t="n">
@@ -3308,22 +3304,22 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>21 g</t>
+          <t>94 g</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>Bambu ASA 1 kg (enclosed printer)</t>
+          <t>Bambu PLA-CF 1 kg (hardened-steel nozzle)</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>Bambu ASA 1 kg (enclosed printer)</t>
+          <t>Bambu PLA-CF 1 kg (hardened-steel nozzle)</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr">
         <is>
-          <t>Tail module F3</t>
+          <t>Wing halves WR/WL (2 walls, 8 % gyroid)</t>
         </is>
       </c>
       <c r="I65" s="4" t="inlineStr">
@@ -3339,7 +3335,7 @@
     </row>
     <row r="66">
       <c r="A66" s="7" t="n">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
@@ -3348,45 +3344,141 @@
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
+          <t>Filament PETG-CF</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>55 g</t>
+        </is>
+      </c>
+      <c r="F66" s="8" t="inlineStr">
+        <is>
+          <t>Bambu PETG-CF 1 kg (hardened-steel nozzle)</t>
+        </is>
+      </c>
+      <c r="G66" s="8" t="inlineStr">
+        <is>
+          <t>Bambu PETG-CF 1 kg (hardened-steel nozzle)</t>
+        </is>
+      </c>
+      <c r="H66" s="8" t="inlineStr">
+        <is>
+          <t>Ailerons, equipment tray, tail coupler, nut bars, hatch lips, duct inserts, motor plate, spinner</t>
+        </is>
+      </c>
+      <c r="I66" s="7" t="inlineStr">
+        <is>
+          <t>Bambu profile</t>
+        </is>
+      </c>
+      <c r="J66" s="8" t="inlineStr">
+        <is>
+          <t>C6B per-part filaments (design/MATERIALS-NOTES.md); one aircraft with the N0M nose</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="n">
+        <v>87</v>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Consumables</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>Filament ASA</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>21 g</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>Bambu ASA 1 kg (enclosed printer)</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>Bambu ASA 1 kg (enclosed printer)</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>Tail module F3</t>
+        </is>
+      </c>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>Bambu profile</t>
+        </is>
+      </c>
+      <c r="J67" s="5" t="inlineStr">
+        <is>
+          <t>C6B per-part filaments (design/MATERIALS-NOTES.md); one aircraft with the N0M nose</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="n">
+        <v>88</v>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Consumables</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
           <t>Filament PETG</t>
         </is>
       </c>
-      <c r="D66" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E66" s="7" t="inlineStr">
-        <is>
-          <t>21 g</t>
-        </is>
-      </c>
-      <c r="F66" s="8" t="inlineStr">
+      <c r="D68" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>20 g</t>
+        </is>
+      </c>
+      <c r="F68" s="8" t="inlineStr">
         <is>
           <t>Bambu PETG Basic 1 kg</t>
         </is>
       </c>
-      <c r="G66" s="8" t="inlineStr">
+      <c r="G68" s="8" t="inlineStr">
         <is>
           <t>Bambu PETG Basic 1 kg</t>
         </is>
       </c>
-      <c r="H66" s="8" t="inlineStr">
+      <c r="H68" s="8" t="inlineStr">
         <is>
           <t>Camera noses, VTX shelf, hatch cover, GPS carrier</t>
         </is>
       </c>
-      <c r="I66" s="7" t="inlineStr">
+      <c r="I68" s="7" t="inlineStr">
         <is>
           <t>Bambu profile</t>
         </is>
       </c>
-      <c r="J66" s="8" t="inlineStr">
+      <c r="J68" s="8" t="inlineStr">
         <is>
           <t>C6B per-part filaments (design/MATERIALS-NOTES.md); one aircraft with the N0M nose</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J66"/>
+  <autoFilter ref="A4:J68"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId2"/>
@@ -3394,7 +3486,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3608,7 +3700,7 @@
         <v>4.3</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>1.4</v>
+        <v>1.42</v>
       </c>
       <c r="E10" s="7" t="n">
         <v>2</v>
@@ -3631,10 +3723,10 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>0.47</v>
+        <v>0.33</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>2</v>
@@ -3657,10 +3749,10 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>17.2</v>
+        <v>17.8</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>0.8</v>
+        <v>0.82</v>
       </c>
       <c r="E12" s="7" t="n">
         <v>2</v>
@@ -3683,10 +3775,10 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0.44</v>
+        <v>0.48</v>
       </c>
       <c r="E13" s="4" t="n">
         <v>2</v>
@@ -3761,10 +3853,10 @@
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="E16" s="7" t="n">
         <v>2</v>
@@ -3787,10 +3879,10 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>0.17</v>
+        <v>0.2</v>
       </c>
       <c r="E17" s="4" t="n">
         <v>2</v>
@@ -3865,7 +3957,7 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>47</v>
+        <v>47.2</v>
       </c>
       <c r="D20" s="7" t="n">
         <v>2.98</v>
@@ -3891,10 +3983,10 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>47</v>
+        <v>47.3</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>2.96</v>
+        <v>3</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>2</v>
@@ -4194,7 +4286,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>One aircraft (one aircraft with the N0M nose; N0P is an alternative part): 188.9 g, 20.1 h of printing.</t>
+          <t>One aircraft (one aircraft with the N0M nose; N0P is an alternative part): 190.8 g, 20.1 h of printing.</t>
         </is>
       </c>
     </row>

</xml_diff>